<commit_message>
fix: zero Available cells in org workbooks
</commit_message>
<xml_diff>
--- a/data/xlsx/aeosib--boiler-operation-and-maintenance.xlsx
+++ b/data/xlsx/aeosib--boiler-operation-and-maintenance.xlsx
@@ -136,7 +136,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -223,6 +223,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -623,7 +626,9 @@
       <c r="C16" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="D16" s="27" t="n"/>
+      <c r="D16" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="E16" s="27" t="n">
         <v>10</v>
       </c>
@@ -645,7 +650,9 @@
       <c r="C17" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="D17" s="27" t="n"/>
+      <c r="D17" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="E17" s="27" t="n">
         <v>8</v>
       </c>
@@ -667,7 +674,9 @@
       <c r="C18" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="D18" s="27" t="n"/>
+      <c r="D18" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="E18" s="27" t="n">
         <v>7</v>
       </c>
@@ -689,7 +698,9 @@
       <c r="C19" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="D19" s="27" t="n"/>
+      <c r="D19" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="E19" s="27" t="n">
         <v>8</v>
       </c>
@@ -711,7 +722,9 @@
       <c r="C20" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="D20" s="27" t="n"/>
+      <c r="D20" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="E20" s="27" t="n">
         <v>7</v>
       </c>
@@ -734,7 +747,9 @@
       <c r="C21" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="D21" s="27" t="n"/>
+      <c r="D21" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="E21" s="27" t="n">
         <v>5</v>
       </c>
@@ -756,7 +771,9 @@
       <c r="C22" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="D22" s="27" t="n"/>
+      <c r="D22" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="E22" s="27" t="n">
         <v>5</v>
       </c>
@@ -778,7 +795,9 @@
       <c r="C23" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="D23" s="27" t="n"/>
+      <c r="D23" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="E23" s="27" t="n">
         <v>5</v>
       </c>
@@ -800,7 +819,9 @@
       <c r="C24" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="D24" s="27" t="n"/>
+      <c r="D24" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="E24" s="27" t="n">
         <v>5</v>
       </c>
@@ -822,7 +843,9 @@
       <c r="C25" s="27" t="n">
         <v>2</v>
       </c>
-      <c r="D25" s="27" t="n"/>
+      <c r="D25" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="E25" s="27" t="n">
         <v>5</v>
       </c>
@@ -844,7 +867,9 @@
       <c r="C26" s="27" t="n">
         <v>2</v>
       </c>
-      <c r="D26" s="27" t="n"/>
+      <c r="D26" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="E26" s="27" t="n">
         <v>4</v>
       </c>
@@ -866,7 +891,9 @@
       <c r="C27" s="27" t="n">
         <v>2</v>
       </c>
-      <c r="D27" s="27" t="n"/>
+      <c r="D27" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="E27" s="27" t="n">
         <v>4</v>
       </c>
@@ -888,7 +915,9 @@
       <c r="C28" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="D28" s="27" t="n"/>
+      <c r="D28" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="E28" s="27" t="n">
         <v>4</v>
       </c>
@@ -910,7 +939,9 @@
       <c r="C29" s="27" t="n">
         <v>10</v>
       </c>
-      <c r="D29" s="27" t="n"/>
+      <c r="D29" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="E29" s="27" t="n">
         <v>6</v>
       </c>
@@ -932,7 +963,9 @@
       <c r="C30" s="27" t="n">
         <v>2</v>
       </c>
-      <c r="D30" s="27" t="n"/>
+      <c r="D30" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="E30" s="27" t="n">
         <v>5</v>
       </c>
@@ -954,7 +987,9 @@
       <c r="C31" s="27" t="n">
         <v>2</v>
       </c>
-      <c r="D31" s="27" t="n"/>
+      <c r="D31" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="E31" s="27" t="n">
         <v>4</v>
       </c>
@@ -980,7 +1015,9 @@
       <c r="C32" s="27" t="n">
         <v>2</v>
       </c>
-      <c r="D32" s="27" t="n"/>
+      <c r="D32" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="E32" s="27" t="n">
         <v>3</v>
       </c>
@@ -1002,7 +1039,9 @@
       <c r="C33" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="D33" s="27" t="n"/>
+      <c r="D33" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="E33" s="27" t="n">
         <v>4</v>
       </c>
@@ -1024,7 +1063,9 @@
       <c r="C34" s="27" t="n">
         <v>2</v>
       </c>
-      <c r="D34" s="27" t="n"/>
+      <c r="D34" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="E34" s="27" t="n">
         <v>3</v>
       </c>
@@ -1046,7 +1087,9 @@
       <c r="C35" s="27" t="n">
         <v>2</v>
       </c>
-      <c r="D35" s="27" t="n"/>
+      <c r="D35" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="E35" s="27" t="n">
         <v>3</v>
       </c>
@@ -1068,7 +1111,9 @@
       <c r="C36" s="27" t="n">
         <v>5</v>
       </c>
-      <c r="D36" s="27" t="n"/>
+      <c r="D36" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="E36" s="27" t="n">
         <v>3</v>
       </c>
@@ -1090,7 +1135,9 @@
       <c r="C37" s="27" t="n">
         <v>2</v>
       </c>
-      <c r="D37" s="27" t="n"/>
+      <c r="D37" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="E37" s="27" t="n">
         <v>4</v>
       </c>
@@ -1116,7 +1163,9 @@
       <c r="C38" s="27" t="n">
         <v>2</v>
       </c>
-      <c r="D38" s="27" t="n"/>
+      <c r="D38" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="E38" s="27" t="n">
         <v>5</v>
       </c>
@@ -1138,7 +1187,9 @@
       <c r="C39" s="27" t="n">
         <v>2</v>
       </c>
-      <c r="D39" s="27" t="n"/>
+      <c r="D39" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="E39" s="27" t="n">
         <v>4</v>
       </c>
@@ -1164,7 +1215,9 @@
       <c r="C40" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="D40" s="27" t="n"/>
+      <c r="D40" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="E40" s="27" t="n">
         <v>6</v>
       </c>

</xml_diff>